<commit_message>
Daily listing check 2026-10-05
Treat 'Goalkeeper Home/Away' names as goalkeeper kits.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0149ELLgZdjaY7wRsdGLp26m
</commit_message>
<xml_diff>
--- a/listing-monitor/reports/2026-10-05/qa_2026-10-05.xlsx
+++ b/listing-monitor/reports/2026-10-05/qa_2026-10-05.xlsx
@@ -8,11 +8,15 @@
   </bookViews>
   <sheets>
     <sheet name="Tổng quan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="RFK" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cần xác nhận" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="RFS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="RFK" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CFS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Cần xác nhận" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RFK'!$A$1:$N$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RFS'!$A$1:$N$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RFK'!$A$1:$N$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CFS'!$A$1:$N$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -478,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tạo lúc 2026-10-05 08:04. Mức độ: Cao = sai thông tin / gây confuse khách và Google; Trung bình = cần sửa; Thấp = nên sửa.</t>
+          <t>Tạo lúc 2026-10-05 22:28. Mức độ: Cao = sai thông tin / gây confuse khách và Google; Trung bình = cần sửa; Thấp = nên sửa.</t>
         </is>
       </c>
     </row>
@@ -522,14 +526,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RFK</t>
+          <t>RFS</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C5" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -538,139 +542,280 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>16</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RFK</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>17</v>
+      </c>
+      <c r="C6" t="n">
+        <v>17</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>19</v>
+      </c>
+      <c r="G6" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CFS</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Số listing bị lỗi theo nhóm</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Nhóm lỗi</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>RFS</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>RFK</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>CFS</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Tổng</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Words to Avoid</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>13</v>
-      </c>
-      <c r="C9" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>SEO</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>11</v>
-      </c>
-      <c r="C10" t="n">
-        <v>11</v>
-      </c>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>1</v>
       </c>
       <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
         <v>1</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Sai đối tượng</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" t="n">
+        <v>6</v>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Lỗi lặp lại trên phần lớn listing của 1 site (nhiều khả năng do TEMPLATE, sửa template 1 lần)</t>
-        </is>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="n">
+        <v>17</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Nhóm</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Vị trí</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Lỗi</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Số listing</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>15</v>
+      </c>
+      <c r="D14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Lỗi lặp lại trên phần lớn listing của 1 site (nhiều khả năng do TEMPLATE, sửa template 1 lần)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Nhóm</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Vị trí</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Lỗi</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Số listing</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CFS</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Sai đối tượng</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Bảng size</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Bảng size trong description có ['3XL', '4XL'] nhưng không mu</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>6/8</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>RFK</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Words to Avoid</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Short description</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>'Trustpilot'</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>13/13</t>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>17/17</t>
         </is>
       </c>
     </row>
@@ -685,7 +830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -784,6 +929,531 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>2026-10-05 16:32</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>104401</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>RFS_LU_AW/THGP_KD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Leeds United 2026/27 Gift Bundle – Away and Third Fan-Version Kids Football Kits</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Short description</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>'Trustpilot' (★ Rated 4.9 on Trustpilot By 100+ customers ✈ Fully Tra...)</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://replicafootballshirt.com/product/leeds-united-2026-27-gift-bundle-away-and-third-fan-version-kids-football-kits/</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-05 16:47</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>104418</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>RFS_ENG_HODADSON_AD/KD_No_2026</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Spain World Cup 2026 Gift Bundle – Home Dad Shirt and Son Kit Fan-Version</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Mã đối tượng trong SKU không rõ: AD/KD</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Dùng AD / KD / WM / ADK / BABY</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://replicafootballshirt.com/product/spain-world-cup-2026-gift-bundle-home-dad-shirt-and-son-kit-fan-version/</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-05 16:47</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>104418</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>RFS_ENG_HODADSON_AD/KD_No_2026</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Spain World Cup 2026 Gift Bundle – Home Dad Shirt and Son Kit Fan-Version</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Short description</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>'Trustpilot' (★ Rated 4.9 on Trustpilot By 100+ customers ✈ Fully Tra...)</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://replicafootballshirt.com/product/spain-world-cup-2026-gift-bundle-home-dad-shirt-and-son-kit-fan-version/</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-05 16:32</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>104401</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>RFS_LU_AW/THGP_KD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Leeds United 2026/27 Gift Bundle – Away and Third Fan-Version Kids Football Kits</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>SEO title</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>SEO title dài 116 ký tự (nên &lt;= 60)</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://replicafootballshirt.com/product/leeds-united-2026-27-gift-bundle-away-and-third-fan-version-kids-football-kits/</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-05 16:32</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>104401</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>RFS_LU_AW/THGP_KD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Leeds United 2026/27 Gift Bundle – Away and Third Fan-Version Kids Football Kits</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Meta description</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Meta dài 199 ký tự (nên &lt;= 160)</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://replicafootballshirt.com/product/leeds-united-2026-27-gift-bundle-away-and-third-fan-version-kids-football-kits/</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-05 16:32</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>104401</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>RFS_LU_AW/THGP_KD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Leeds United 2026/27 Gift Bundle – Away and Third Fan-Version Kids Football Kits</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Meta description</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>có ký tự &amp; hoặc ": "Celebrate Birthday in true football style with the Leeds United 2026/27 Gift Bundle – Away and Third Fan-Version Kids Football Kits – featuring Away &amp; Third Replica Kits. Perfect gift for young fans."</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Sửa định dạng</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://replicafootballshirt.com/product/leeds-united-2026-27-gift-bundle-away-and-third-fan-version-kids-football-kits/</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-05 16:47</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>104418</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>RFS_ENG_HODADSON_AD/KD_No_2026</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Spain World Cup 2026 Gift Bundle – Home Dad Shirt and Son Kit Fan-Version</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>SEO title</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>SEO title dài 109 ký tự (nên &lt;= 60)</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://replicafootballshirt.com/product/spain-world-cup-2026-gift-bundle-home-dad-shirt-and-son-kit-fan-version/</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N8"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId14"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Mức độ</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Ngày đăng</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Tên sản phẩm</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Nhóm lỗi</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Vị trí</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Chi tiết</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Cách sửa</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Lỗi template?</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Sửa trong admin</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Người sửa</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Đã sửa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>2026-10-05 06:48</t>
         </is>
       </c>
@@ -1821,57 +2491,53 @@
       <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-05 05:21</t>
+          <t>2026-10-05 08:14</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>127452</v>
+        <v>127690</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>RFK_BA_TH_AD_No_98/99</t>
+          <t>RFK_BA_AW_AD_No_14/15</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Retro Barcelona Third Men Replica Football Shirt 1998/99</t>
+          <t>Retro Barcelona Away Men Replica Football Shirt 2014/15</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Short description</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+          <t>SEO title dài 72 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/retro-brclna-third-men-replica-football-shirt-1998-99/</t>
+          <t>https://replicafootballkits.com/product/retro-brclna-away-men-replica-football-shirt-2014-15/</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -1883,57 +2549,53 @@
       <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-05 06:10</t>
+          <t>2026-10-05 08:22</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>127489</v>
+        <v>127702</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>RFK_ENG_HO_AD_No_2016</t>
+          <t>RFK_RM_TH_AD_No_10/11</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Retro England Home Men Replica Football Shirt 2016</t>
+          <t>Retro Real Madrid Third Replica Football Shirt 2010/11</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Short description</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+          <t>SEO title dài 71 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/retro-e-n-home-men-replica-football-shirt-2016/</t>
+          <t>https://replicafootballkits.com/product/retro-rl-md-third-replica-football-shirt-2010-11/</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -1945,57 +2607,53 @@
       <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-05 06:23</t>
+          <t>2026-10-05 10:14</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>127501</v>
+        <v>127792</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>RFK_AL_HO_AD_No_26/27</t>
+          <t>RFK_POR_AW_AD_No_2016</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Al Hilal Home Men Replica Football Shirt 2026/27</t>
+          <t>Retro Portugal Away Men Replica Football Shirt 2016</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Short description</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+          <t>SEO title dài 68 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/al-hilal-home-men-replica-football-shirt-2026-27/</t>
+          <t>https://replicafootballkits.com/product/retro-por-away-men-replica-football-shirt-2016/</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -2007,57 +2665,53 @@
       <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-05 06:30</t>
+          <t>2026-10-05 10:18</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>127516</v>
+        <v>127806</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>RFK_AL_AW_AD_No_26/27</t>
+          <t>RFK_POR_AWLS_AD_No_2016</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Al Hilal Away Men Replica Football Shirt 2026/27</t>
+          <t>Retro Portugal Away Men Replica Football Shirt 2016 Long Sleeve</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Short description</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+          <t>SEO title dài 80 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/al-hilal-away-men-replica-football-shirt-2026-27/</t>
+          <t>https://replicafootballkits.com/product/retro-por-away-men-replica-football-shirt-2016-long-sleeve/</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -2069,57 +2723,53 @@
       <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-05 06:48</t>
+          <t>2026-10-05 10:18</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>127535</v>
+        <v>127806</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>RFK_POR_AW_AD_No_2015</t>
+          <t>RFK_POR_AWLS_AD_No_2016</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Retro Portugal Away Men Replica Football Shirt 2015</t>
+          <t>Retro Portugal Away Men Replica Football Shirt 2016 Long Sleeve</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Short description</t>
+          <t>Meta description</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+          <t>Meta dài 170 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/retro-por-away-men-replica-football-shirt-2015/</t>
+          <t>https://replicafootballkits.com/product/retro-por-away-men-replica-football-shirt-2016-long-sleeve/</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr">
@@ -2138,20 +2788,20 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-05 06:58</t>
+          <t>2026-10-05 05:21</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>127547</v>
+        <v>127452</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>RFK_POR_HO_AD_No_2018</t>
+          <t>RFK_BA_TH_AD_No_98/99</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Retro Portugal Home Men Replica Football Shirt 2018</t>
+          <t>Retro Barcelona Third Men Replica Football Shirt 1998/99</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2181,7 +2831,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/retro-por-home-men-replica-football-shirt-2018/</t>
+          <t>https://replicafootballkits.com/product/retro-brclna-third-men-replica-football-shirt-1998-99/</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -2200,20 +2850,20 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-05 07:09</t>
+          <t>2026-10-05 06:10</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>127560</v>
+        <v>127489</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>RFK_POR_HOLS_AD_No_2018</t>
+          <t>RFK_ENG_HO_AD_No_2016</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Retro Portugal Home Men Replica Football Shirt 2018 Long Sleeve</t>
+          <t>Retro England Home Men Replica Football Shirt 2016</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2243,7 +2893,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/retro-por-home-men-replica-football-shirt-2018-long-sleeve/</t>
+          <t>https://replicafootballkits.com/product/retro-e-n-home-men-replica-football-shirt-2016/</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
@@ -2262,20 +2912,20 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-05 07:17</t>
+          <t>2026-10-05 06:23</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>127572</v>
+        <v>127501</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>RFK_POR_HO_AD_No_2012</t>
+          <t>RFK_AL_HO_AD_No_26/27</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Retro Portugal Home Men Replica Football Shirt 2012</t>
+          <t>Al Hilal Home Men Replica Football Shirt 2026/27</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2305,7 +2955,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/retro-por-home-men-replica-football-shirt-2012/</t>
+          <t>https://replicafootballkits.com/product/al-hilal-home-men-replica-football-shirt-2026-27/</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
@@ -2324,20 +2974,20 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-10-05 07:21</t>
+          <t>2026-10-05 06:30</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>127587</v>
+        <v>127516</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>RFK_POR_HOLS_AD_No_2012</t>
+          <t>RFK_AL_AW_AD_No_26/27</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Retro Portugal Home Men Replica Football Shirt 2012 Long Sleeve</t>
+          <t>Al Hilal Away Men Replica Football Shirt 2026/27</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2367,7 +3017,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/retro-por-home-men-replica-football-shirt-2012-long-sleeve/</t>
+          <t>https://replicafootballkits.com/product/al-hilal-away-men-replica-football-shirt-2026-27/</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr">
@@ -2386,20 +3036,20 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-10-05 07:26</t>
+          <t>2026-10-05 06:48</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>127596</v>
+        <v>127535</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>RFK_POR_AW_AD_No_2012</t>
+          <t>RFK_POR_AW_AD_No_2015</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Retro Portugal Away Men Replica Football Shirt 2012</t>
+          <t>Retro Portugal Away Men Replica Football Shirt 2015</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2429,7 +3079,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/retro-por-away-men-replica-football-shirt-2012/</t>
+          <t>https://replicafootballkits.com/product/retro-por-away-men-replica-football-shirt-2015/</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr">
@@ -2448,20 +3098,20 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-10-05 07:32</t>
+          <t>2026-10-05 06:58</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>127611</v>
+        <v>127547</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>RFK_POR_AWLS_AD_No_2012</t>
+          <t>RFK_POR_HO_AD_No_2018</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Retro Portugal Away Men Replica Football Shirt 2012 Long Sleeve</t>
+          <t>Retro Portugal Home Men Replica Football Shirt 2018</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2491,7 +3141,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/retro-por-away-men-replica-football-shirt-2012-long-sleeve/</t>
+          <t>https://replicafootballkits.com/product/retro-por-home-men-replica-football-shirt-2018/</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr">
@@ -2510,20 +3160,20 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-10-05 07:38</t>
+          <t>2026-10-05 07:09</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>127621</v>
+        <v>127560</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>RFK_POR_HO_AD_No_2016</t>
+          <t>RFK_POR_HOLS_AD_No_2018</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Retro Portugal Home Men Replica Football Shirt 2016</t>
+          <t>Retro Portugal Home Men Replica Football Shirt 2018 Long Sleeve</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2553,7 +3203,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/retro-por-home-men-replica-football-shirt-2016/</t>
+          <t>https://replicafootballkits.com/product/retro-por-home-men-replica-football-shirt-2018-long-sleeve/</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr">
@@ -2572,20 +3222,20 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-10-05 07:44</t>
+          <t>2026-10-05 07:17</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>127636</v>
+        <v>127572</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>RFK_POR_HOLS_AD_No_2016</t>
+          <t>RFK_POR_HO_AD_No_2012</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Retro Portugal Home Men Replica Football Shirt 2016 Long Sleeve</t>
+          <t>Retro Portugal Home Men Replica Football Shirt 2012</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2615,7 +3265,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/retro-por-home-men-replica-football-shirt-2016-long-sleeve/</t>
+          <t>https://replicafootballkits.com/product/retro-por-home-men-replica-football-shirt-2012/</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr">
@@ -2626,8 +3276,566 @@
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
     </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-10-05 07:21</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>127587</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>RFK_POR_HOLS_AD_No_2012</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Retro Portugal Home Men Replica Football Shirt 2012 Long Sleeve</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Short description</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>https://replicafootballkits.com/product/retro-por-home-men-replica-football-shirt-2012-long-sleeve/</t>
+        </is>
+      </c>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-10-05 07:26</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>127596</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>RFK_POR_AW_AD_No_2012</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Retro Portugal Away Men Replica Football Shirt 2012</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Short description</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>https://replicafootballkits.com/product/retro-por-away-men-replica-football-shirt-2012/</t>
+        </is>
+      </c>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-10-05 07:32</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>127611</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>RFK_POR_AWLS_AD_No_2012</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Retro Portugal Away Men Replica Football Shirt 2012 Long Sleeve</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Short description</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>https://replicafootballkits.com/product/retro-por-away-men-replica-football-shirt-2012-long-sleeve/</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-10-05 07:38</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>127621</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>RFK_POR_HO_AD_No_2016</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Retro Portugal Home Men Replica Football Shirt 2016</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Short description</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>https://replicafootballkits.com/product/retro-por-home-men-replica-football-shirt-2016/</t>
+        </is>
+      </c>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-10-05 07:44</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>127636</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>RFK_POR_HOLS_AD_No_2016</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Retro Portugal Home Men Replica Football Shirt 2016 Long Sleeve</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Short description</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>https://replicafootballkits.com/product/retro-por-home-men-replica-football-shirt-2016-long-sleeve/</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-10-05 08:14</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>127690</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>RFK_BA_AW_AD_No_14/15</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Retro Barcelona Away Men Replica Football Shirt 2014/15</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Short description</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>https://replicafootballkits.com/product/retro-brclna-away-men-replica-football-shirt-2014-15/</t>
+        </is>
+      </c>
+      <c r="L38" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-10-05 08:22</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>127702</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>RFK_RM_TH_AD_No_10/11</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Retro Real Madrid Third Replica Football Shirt 2010/11</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Short description</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>https://replicafootballkits.com/product/retro-rl-md-third-replica-football-shirt-2010-11/</t>
+        </is>
+      </c>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:14</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>127792</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>RFK_POR_AW_AD_No_2016</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Retro Portugal Away Men Replica Football Shirt 2016</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Short description</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>https://replicafootballkits.com/product/retro-por-away-men-replica-football-shirt-2016/</t>
+        </is>
+      </c>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:18</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>127806</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>RFK_POR_AWLS_AD_No_2016</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Retro Portugal Away Men Replica Football Shirt 2016 Long Sleeve</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Short description</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>https://replicafootballkits.com/product/retro-por-away-men-replica-football-shirt-2016-long-sleeve/</t>
+        </is>
+      </c>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N32"/>
+  <autoFilter ref="A1:N41"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
@@ -2691,12 +3899,1299 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId80"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Mức độ</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Ngày đăng</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Tên sản phẩm</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Nhóm lỗi</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Vị trí</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Chi tiết</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Cách sửa</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Lỗi template?</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Sửa trong admin</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Người sửa</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Đã sửa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:58</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>82785</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CFS_HC_GK_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Hull City Goalkeeper Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>'Showcases the' (...es. Football-Inspired Design: Showcases the iconic diagonal chest detail ...)</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Showcases the -&gt; includes the / highlights the</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/hull-city-goalkeeper-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:35</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>82815</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CFS_WOL_TH_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Wolves Third Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Words to Avoid</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>'Showcases the' (...ve. Football-Inspired Design: Showcases the iconic wolf head chest detail...)</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Showcases the -&gt; includes the / highlights the</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/wolves-third-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:58</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>82785</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CFS_HC_GK_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Hull City Goalkeeper Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Meta description</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Meta dài 176 ký tự (nên &lt;= 160)</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/hull-city-goalkeeper-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-05 14:06</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>82791</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CFS_DBC_TH_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Derby County Third Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Meta description</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Meta dài 166 ký tự (nên &lt;= 160)</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/derby-county-third-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-05 14:06</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>82791</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CFS_DBC_TH_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Derby County Third Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Meta description</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>khoảng trắng trước dấu câu: "Get the Derby County Third Men Cheap Football Shirt 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Sửa định dạng</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/derby-county-third-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:14</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>82797</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CFS_NC_GreenGK_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Newcastle United Green Goalkeeper Home Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>SEO title</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>SEO title dài 71 ký tự (nên &lt;= 60)</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/newcastle-united-green-goalkeeper-home-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:14</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>82797</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>CFS_NC_GreenGK_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Newcastle United Green Goalkeeper Home Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Meta description</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Meta dài 193 ký tự (nên &lt;= 160)</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/newcastle-united-green-goalkeeper-home-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:23</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>82803</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>CFS_BM_AW_WM_No_26/27</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Bayern Munich Away Women Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Meta description</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Meta dài 176 ký tự (nên &lt;= 160)</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/bayern-munich-away-women-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:30</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>82809</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CFS_BM_HO_WM_No_26/27</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Bayern Munich Home Women Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Meta description</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Meta dài 176 ký tự (nên &lt;= 160)</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/bayern-munich-home-women-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:35</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>82815</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>CFS_WOL_TH_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Wolves Third Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Meta description</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Meta dài 168 ký tự (nên &lt;= 160)</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/wolves-third-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:44</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>82821</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>CFS_SHU_TH_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Sheffield United Third Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Meta description</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Meta dài 178 ký tự (nên &lt;= 160)</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/sheffield-united-third-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:59</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>82833</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>CFS_BM_TN_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Bayern Munich Training Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Meta description</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Meta dài 170 ký tự (nên &lt;= 160)</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/bayern-munich-training-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:59</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>82833</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>CFS_BM_TN_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Bayern Munich Training Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Meta description</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>khoảng trắng trước dấu câu: "Get the Bayern Munich Training Men Cheap Football Shirt 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Sửa định dạng</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/bayern-munich-training-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-05 13:58</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>82785</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CFS_HC_GK_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Hull City Goalkeeper Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Sai đối tượng</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Bảng size</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Bảng size trong description có ['3XL', '4XL'] nhưng không mua được (size đang bán: ['L', 'M', 'S', 'XL', 'XXL'])</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Bỏ dòng size không bán khỏi bảng, hoặc thêm variation</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/hull-city-goalkeeper-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-10-05 14:06</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>82791</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CFS_DBC_TH_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Derby County Third Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Sai đối tượng</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Bảng size</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Bảng size trong description có ['3XL', '4XL'] nhưng không mua được (size đang bán: ['L', 'M', 'S', 'XL', 'XXL'])</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Bỏ dòng size không bán khỏi bảng, hoặc thêm variation</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/derby-county-third-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:14</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>82797</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>CFS_NC_GreenGK_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Newcastle United Green Goalkeeper Home Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Sai đối tượng</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Bảng size</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Bảng size trong description có ['3XL', '4XL'] nhưng không mua được (size đang bán: ['L', 'M', 'S', 'XL', 'XXL'])</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Bỏ dòng size không bán khỏi bảng, hoặc thêm variation</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/newcastle-united-green-goalkeeper-home-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:35</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>82815</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CFS_WOL_TH_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Wolves Third Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Sai đối tượng</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Bảng size</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Bảng size trong description có ['3XL', '4XL'] nhưng không mua được (size đang bán: ['L', 'M', 'S', 'XL', 'XXL'])</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Bỏ dòng size không bán khỏi bảng, hoặc thêm variation</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/wolves-third-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:44</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>82821</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CFS_SHU_TH_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Sheffield United Third Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Sai đối tượng</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Bảng size</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Bảng size trong description có ['3XL', '4XL'] nhưng không mua được (size đang bán: ['L', 'M', 'S', 'XL', 'XXL'])</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Bỏ dòng size không bán khỏi bảng, hoặc thêm variation</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/sheffield-united-third-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:59</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>82833</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>CFS_BM_TN_AD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Bayern Munich Training Men Cheap Football Shirt 2026/27</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Sai đối tượng</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Bảng size</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Bảng size trong description có ['3XL', '4XL'] nhưng không mua được (size đang bán: ['L', 'M', 'S', 'XL', 'XXL'])</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Bỏ dòng size không bán khỏi bảng, hoặc thêm variation</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/bayern-munich-training-men-cheap-football-shirt-2026-27/</t>
+        </is>
+      </c>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N20"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId38"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>